<commit_message>
first round, code breaks down might be due to the synthetic data
</commit_message>
<xml_diff>
--- a/package-output-map.xlsx
+++ b/package-output-map.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10609"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29127"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/floswald/git/JPEtemplate/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\bz.ad.minbuza.local\Data\users\broos.nafthali\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{067DD2C7-24FE-2447-A5A8-8F6542C7C06E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="14_{FC72D6C1-CAE1-4C2E-9B83-773915727E83}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="760" windowWidth="21900" windowHeight="12060" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="28680" yWindow="-2610" windowWidth="29040" windowHeight="15720" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="11" uniqueCount="7">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="120" uniqueCount="62">
   <si>
     <t>Data Preparation Program</t>
   </si>
@@ -42,17 +42,182 @@
     <t>Program</t>
   </si>
   <si>
-    <t>Line Number</t>
-  </si>
-  <si>
-    <t>In-text numbers</t>
+    <t>Figure 1</t>
+  </si>
+  <si>
+    <t>code/explore_numerator/plot_market_shares.R</t>
+  </si>
+  <si>
+    <t>No</t>
+  </si>
+  <si>
+    <t>Figure 2</t>
+  </si>
+  <si>
+    <t>code/describe_portfolio_choice/describe_portfolio_choice.R</t>
+  </si>
+  <si>
+    <t>Figure 3</t>
+  </si>
+  <si>
+    <t>code/CF/analyze_vary_cap.R</t>
+  </si>
+  <si>
+    <t>Figure 4a-c</t>
+  </si>
+  <si>
+    <t>Figure 5</t>
+  </si>
+  <si>
+    <t>code/CF/variety_vs_fixed_costs.R</t>
+  </si>
+  <si>
+    <t>Figure 6a-b</t>
+  </si>
+  <si>
+    <t>code/CF/relative_change_plot_take2.R</t>
+  </si>
+  <si>
+    <t>Figure 7</t>
+  </si>
+  <si>
+    <t>code/CF/analyze_twosided.R</t>
+  </si>
+  <si>
+    <t>Figure 8a-c</t>
+  </si>
+  <si>
+    <t>Table 1</t>
+  </si>
+  <si>
+    <t>code/explore_yipit/process_demand_estimation_DiD.R</t>
+  </si>
+  <si>
+    <t>Table 2</t>
+  </si>
+  <si>
+    <t>code/demand_estimation/produce_table.R</t>
+  </si>
+  <si>
+    <t>Table 3a</t>
+  </si>
+  <si>
+    <t>code/recover_restaurant_costs/summarize_costs_v3.R</t>
+  </si>
+  <si>
+    <t>Table 3b</t>
+  </si>
+  <si>
+    <t>Table 4a-c</t>
+  </si>
+  <si>
+    <t>code/restaurant_FC_estimation/GMM_CCP_table.R</t>
+  </si>
+  <si>
+    <t>Table 5</t>
+  </si>
+  <si>
+    <t>code/estimate_platform_costs/describe_pMC.R</t>
+  </si>
+  <si>
+    <t>Table 6</t>
+  </si>
+  <si>
+    <t>code/CF/compare_priv_soc.R</t>
+  </si>
+  <si>
+    <t>Table 7</t>
+  </si>
+  <si>
+    <t>code/CF/compute_distortions.R</t>
+  </si>
+  <si>
+    <t>Table 8a-b</t>
+  </si>
+  <si>
+    <t>Appendix Table A1</t>
+  </si>
+  <si>
+    <t>code/numerator_menu_pricing/generate_item_level_reg_table.R</t>
+  </si>
+  <si>
+    <t>OA Tables/Figures</t>
+  </si>
+  <si>
+    <t>various</t>
+  </si>
+  <si>
+    <t>Table 9</t>
+  </si>
+  <si>
+    <t>code/CF/variety_vs_fixed_costs_soc_priv.R</t>
+  </si>
+  <si>
+    <t>Table 10</t>
+  </si>
+  <si>
+    <t>code/CF/decompose_rpi_soc_fees.R</t>
+  </si>
+  <si>
+    <t>Table 11</t>
+  </si>
+  <si>
+    <t>Table 12</t>
+  </si>
+  <si>
+    <t>Table 13</t>
+  </si>
+  <si>
+    <t>Table 14a-b</t>
+  </si>
+  <si>
+    <t>code/CF/analyze_max_joint.R</t>
+  </si>
+  <si>
+    <t>Table 15</t>
+  </si>
+  <si>
+    <t>output/explore_yipit/DiD_for_demand_estimation-paper.csv</t>
+  </si>
+  <si>
+    <t>output/demand_estimation/est_SE-yipitdata_formatted.csv</t>
+  </si>
+  <si>
+    <t>output/recover_restaurant_costs/describe/combo_tab_mc_all_SEs.csv</t>
+  </si>
+  <si>
+    <t>output/recover_restaurant_costs/describe/combo_tab_all_SEs.csv</t>
+  </si>
+  <si>
+    <t>output/restaurant_FC_estimation/restaurant_cost_RC_GMM-ccp_sigmas.csv</t>
+  </si>
+  <si>
+    <t>output/restaurant_FC_estimation/restaurant_cost_RC_GMM-ccp_kappas.csv</t>
+  </si>
+  <si>
+    <t>output/estimate_platform_costs/MC_H/spec_nsim50/MC_results.csv</t>
+  </si>
+  <si>
+    <t>output/CF_feefirst/analysis_nsim50/compare_priv_soc_CR.csv</t>
+  </si>
+  <si>
+    <t>output/CF_feefirst/analysis_nsim50/distortions_table.csv</t>
+  </si>
+  <si>
+    <t>output/CF_feefirst/analysis_nsim50/welfare_soc_priv.csv</t>
+  </si>
+  <si>
+    <t>output/CF_feefirst/analysis_nsim50/soc_priv_observables.csv</t>
+  </si>
+  <si>
+    <t>output/numerator_menu_pricing/disagg_results/pricing_reg_combo_allsample.csv</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color rgb="FF000000"/>
@@ -67,6 +232,12 @@
       <name val="Calibri"/>
       <family val="2"/>
       <charset val="1"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF000000"/>
+      <name val="Calibri"/>
+      <family val="2"/>
     </font>
   </fonts>
   <fills count="2">
@@ -89,7 +260,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
@@ -100,9 +271,12 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="Normal" xfId="0" builtinId="0"/>
+    <cellStyle name="Standaard" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -118,7 +292,7 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Kantoorthema">
   <a:themeElements>
     <a:clrScheme name="Office">
       <a:dk1>
@@ -434,22 +608,22 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:D18"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.6640625" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <dimension ref="A1:D41"/>
+  <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="23.5" customWidth="1"/>
-    <col min="2" max="2" width="13.33203125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="23.42578125" customWidth="1"/>
+    <col min="2" max="2" width="38.140625" customWidth="1"/>
     <col min="3" max="3" width="13" customWidth="1"/>
-    <col min="5" max="5" width="12.1640625" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="11.1640625" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="11.5" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="13.5" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="7.6640625" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="11.1640625" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="11.5" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="12.140625" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="11.140625" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="11.42578125" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="13.42578125" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="7.7109375" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="11.140625" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="11.42578125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -460,52 +634,438 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A2" s="3"/>
-      <c r="B2" s="3"/>
-    </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A3" s="3"/>
-      <c r="B3" s="3"/>
-    </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A4" s="3"/>
-      <c r="B4" s="3"/>
-    </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A5" s="3"/>
-      <c r="B5" s="3"/>
-    </row>
-    <row r="10" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A10" s="1" t="s">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A2" s="3" t="s">
+        <v>21</v>
+      </c>
+      <c r="B2" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="C2" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A3" s="3" t="s">
+        <v>23</v>
+      </c>
+      <c r="B3" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="C3" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A4" s="3" t="s">
+        <v>25</v>
+      </c>
+      <c r="B4" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="C4" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A5" s="3" t="s">
+        <v>25</v>
+      </c>
+      <c r="B5" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="C5" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A6" s="3" t="s">
+        <v>28</v>
+      </c>
+      <c r="B6" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="C6" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A7" s="3" t="s">
+        <v>28</v>
+      </c>
+      <c r="B7" s="3" t="s">
+        <v>55</v>
+      </c>
+      <c r="C7" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>30</v>
+      </c>
+      <c r="B8" t="s">
+        <v>56</v>
+      </c>
+      <c r="C8" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
+        <v>32</v>
+      </c>
+      <c r="B9" t="s">
+        <v>57</v>
+      </c>
+      <c r="C9" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="10" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A10" t="s">
+        <v>34</v>
+      </c>
+      <c r="B10" t="s">
+        <v>58</v>
+      </c>
+      <c r="C10" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="11" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A11" t="s">
+        <v>32</v>
+      </c>
+      <c r="B11" t="s">
+        <v>59</v>
+      </c>
+      <c r="C11" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="12" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A12" t="s">
+        <v>32</v>
+      </c>
+      <c r="B12" t="s">
+        <v>60</v>
+      </c>
+      <c r="C12" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="13" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A13" t="s">
+        <v>37</v>
+      </c>
+      <c r="B13" t="s">
+        <v>61</v>
+      </c>
+      <c r="C13" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="15" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A15" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="B10" s="1" t="s">
+      <c r="B15" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="C10" s="1" t="s">
+      <c r="C15" s="2" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="16" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A16" t="s">
         <v>5</v>
       </c>
-      <c r="D10" s="2" t="s">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="18" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A18" s="1" t="s">
+      <c r="B16" t="s">
         <v>6</v>
       </c>
-      <c r="B18" s="1" t="s">
-        <v>4</v>
-      </c>
-      <c r="C18" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="D18" s="2" t="s">
-        <v>2</v>
+      <c r="C16" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="17" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A17" t="s">
+        <v>8</v>
+      </c>
+      <c r="B17" t="s">
+        <v>9</v>
+      </c>
+      <c r="C17" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="18" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A18" t="s">
+        <v>10</v>
+      </c>
+      <c r="B18" t="s">
+        <v>11</v>
+      </c>
+      <c r="C18" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="19" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A19" t="s">
+        <v>12</v>
+      </c>
+      <c r="B19" t="s">
+        <v>11</v>
+      </c>
+      <c r="C19" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="20" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A20" t="s">
+        <v>13</v>
+      </c>
+      <c r="B20" t="s">
+        <v>14</v>
+      </c>
+      <c r="C20" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="21" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A21" t="s">
+        <v>15</v>
+      </c>
+      <c r="B21" t="s">
+        <v>16</v>
+      </c>
+      <c r="C21" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="22" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A22" t="s">
+        <v>17</v>
+      </c>
+      <c r="B22" t="s">
+        <v>18</v>
+      </c>
+      <c r="C22" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="23" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A23" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="B23" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="C23" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="D23" s="2"/>
+    </row>
+    <row r="24" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A24" t="s">
+        <v>20</v>
+      </c>
+      <c r="B24" t="s">
+        <v>21</v>
+      </c>
+      <c r="C24" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="25" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A25" t="s">
+        <v>22</v>
+      </c>
+      <c r="B25" t="s">
+        <v>23</v>
+      </c>
+      <c r="C25" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="26" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A26" t="s">
+        <v>24</v>
+      </c>
+      <c r="B26" t="s">
+        <v>25</v>
+      </c>
+      <c r="C26" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="27" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A27" t="s">
+        <v>26</v>
+      </c>
+      <c r="B27" t="s">
+        <v>25</v>
+      </c>
+      <c r="C27" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="28" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A28" t="s">
+        <v>27</v>
+      </c>
+      <c r="B28" t="s">
+        <v>28</v>
+      </c>
+      <c r="C28" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="29" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A29" t="s">
+        <v>29</v>
+      </c>
+      <c r="B29" t="s">
+        <v>30</v>
+      </c>
+      <c r="C29" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="30" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A30" t="s">
+        <v>31</v>
+      </c>
+      <c r="B30" t="s">
+        <v>32</v>
+      </c>
+      <c r="C30" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="31" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A31" t="s">
+        <v>33</v>
+      </c>
+      <c r="B31" t="s">
+        <v>34</v>
+      </c>
+      <c r="C31" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="32" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A32" t="s">
+        <v>35</v>
+      </c>
+      <c r="B32" t="s">
+        <v>32</v>
+      </c>
+      <c r="C32" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="33" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A33" t="s">
+        <v>40</v>
+      </c>
+      <c r="B33" t="s">
+        <v>41</v>
+      </c>
+      <c r="C33" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="34" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A34" t="s">
+        <v>42</v>
+      </c>
+      <c r="B34" t="s">
+        <v>43</v>
+      </c>
+      <c r="C34" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="35" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A35" t="s">
+        <v>44</v>
+      </c>
+      <c r="B35" t="s">
+        <v>11</v>
+      </c>
+      <c r="C35" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="36" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A36" t="s">
+        <v>45</v>
+      </c>
+      <c r="B36" t="s">
+        <v>11</v>
+      </c>
+      <c r="C36" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="37" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A37" t="s">
+        <v>46</v>
+      </c>
+      <c r="B37" t="s">
+        <v>11</v>
+      </c>
+      <c r="C37" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="38" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A38" t="s">
+        <v>47</v>
+      </c>
+      <c r="B38" t="s">
+        <v>48</v>
+      </c>
+      <c r="C38" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="39" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A39" t="s">
+        <v>49</v>
+      </c>
+      <c r="B39" t="s">
+        <v>48</v>
+      </c>
+      <c r="C39" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="40" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A40" t="s">
+        <v>36</v>
+      </c>
+      <c r="B40" t="s">
+        <v>37</v>
+      </c>
+      <c r="C40" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="41" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A41" t="s">
+        <v>38</v>
+      </c>
+      <c r="B41" t="s">
+        <v>39</v>
+      </c>
+      <c r="C41" t="s">
+        <v>7</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.51180555555555496" footer="0.51180555555555496"/>
-  <pageSetup orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
+  <pageSetup orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>